<commit_message>
Update Additional files 1-5 (consistency fixes)
</commit_message>
<xml_diff>
--- a/manuscript_v2/additional_files/Additional_file_4.xlsx
+++ b/manuscript_v2/additional_files/Additional_file_4.xlsx
@@ -456,7 +456,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Functional categories were assigned to GHB-732 (LR) and GHB-538 (HR) candidates with ONE ordered rule set (sheet 'Rules'), applied identically to both varieties.</t>
+          <t>Functional categories were assigned to GHB-732 (LR) and GHB-538 (HR) candidate genes with ONE ordered rule set (sheet 'Rules'), applied identically to both varieties.</t>
         </is>
       </c>
     </row>
@@ -470,7 +470,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Candidates shared by both varieties were classified from the combined annotation of both sets, so every common gene has the same category in both varieties.</t>
+          <t>Candidate genes shared by both varieties were classified from the combined annotation of both sets, so every common gene has the same category in both varieties.</t>
         </is>
       </c>
     </row>

</xml_diff>